<commit_message>
Adaugă câmp Producător la produse
Câmp opțional producator pe produse, afișat pe pagina produsului și
gestionat din admin.

- worker.js: coloană producator în rowToProduct/upsert/update; ensureSchema
  face ALTER TABLE ADD COLUMN producator (idempotent, auto-migrare)
- schema.sql: coloană producator pentru instalări noi
- admin.html: câmp în editorul de produs, coloană în listă, în save/open și
  în ambele formate de import
- produs.html + style.css: linie „Producător: …" sub titlu
- template-import-produse.xlsx: coloană producator + instrucțiuni

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019PrskwzcAZcS9eQ4XRB5xV
</commit_message>
<xml_diff>
--- a/public/template-import-produse.xlsx
+++ b/public/template-import-produse.xlsx
@@ -513,20 +513,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -569,25 +570,30 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>producator</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>finisaj</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>culoare</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>grosime</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>pret</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>specificatii</t>
         </is>
@@ -626,25 +632,30 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
+          <t>Ruukki</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
           <t>Poliester mat</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Cărămiziu</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>0.50 mm</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>42.90</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>Acoperire: Poliester mat 25µm; Garanție: 15 ani</t>
         </is>
@@ -661,27 +672,28 @@
       <c r="D4" s="7" t="inlineStr"/>
       <c r="E4" s="6" t="inlineStr"/>
       <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>Poliester mat</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>Cărămiziu</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>0.60 mm</t>
         </is>
       </c>
-      <c r="J4" s="8" t="inlineStr">
+      <c r="K4" s="8" t="inlineStr">
         <is>
           <t>51.90</t>
         </is>
       </c>
-      <c r="K4" s="7" t="inlineStr"/>
+      <c r="L4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -694,27 +706,28 @@
       <c r="D5" s="7" t="inlineStr"/>
       <c r="E5" s="6" t="inlineStr"/>
       <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Poliester mat</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>Antracit</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>0.50 mm</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
         <is>
           <t>44.90</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr"/>
+      <c r="L5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -727,27 +740,28 @@
       <c r="D6" s="7" t="inlineStr"/>
       <c r="E6" s="6" t="inlineStr"/>
       <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Poliester mat</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>Antracit</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>0.60 mm</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="K6" s="8" t="inlineStr">
         <is>
           <t>53.90</t>
         </is>
       </c>
-      <c r="K6" s="7" t="inlineStr"/>
+      <c r="L6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -760,27 +774,28 @@
       <c r="D7" s="7" t="inlineStr"/>
       <c r="E7" s="6" t="inlineStr"/>
       <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Mat structurat</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>Cărămiziu</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>0.50 mm</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="K7" s="8" t="inlineStr">
         <is>
           <t>49.90</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -793,27 +808,28 @@
       <c r="D8" s="7" t="inlineStr"/>
       <c r="E8" s="6" t="inlineStr"/>
       <c r="F8" s="6" t="inlineStr"/>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Mat structurat</t>
         </is>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>Cărămiziu</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>0.60 mm</t>
         </is>
       </c>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="K8" s="8" t="inlineStr">
         <is>
           <t>58.90</t>
         </is>
       </c>
-      <c r="K8" s="7" t="inlineStr"/>
+      <c r="L8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -826,27 +842,28 @@
       <c r="D9" s="7" t="inlineStr"/>
       <c r="E9" s="6" t="inlineStr"/>
       <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>Mat structurat</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>Antracit</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>0.50 mm</t>
         </is>
       </c>
-      <c r="J9" s="8" t="inlineStr">
+      <c r="K9" s="8" t="inlineStr">
         <is>
           <t>51.90</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -859,27 +876,28 @@
       <c r="D10" s="7" t="inlineStr"/>
       <c r="E10" s="6" t="inlineStr"/>
       <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Mat structurat</t>
         </is>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>Antracit</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>0.60 mm</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="K10" s="8" t="inlineStr">
         <is>
           <t>60.90</t>
         </is>
       </c>
-      <c r="K10" s="7" t="inlineStr"/>
+      <c r="L10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -910,21 +928,26 @@
       <c r="F11" s="3" t="inlineStr"/>
       <c r="G11" s="3" t="inlineStr">
         <is>
+          <t>Lindab</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
           <t>Lucios</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Antracit</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>23.50</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="L11" s="4" t="inlineStr">
         <is>
           <t>Diametru: 125 mm; Lungime: 3 m</t>
         </is>
@@ -941,27 +964,28 @@
       <c r="D12" s="7" t="inlineStr"/>
       <c r="E12" s="6" t="inlineStr"/>
       <c r="F12" s="6" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Lucios</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>Alb</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr"/>
-      <c r="J12" s="8" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="8" t="inlineStr">
         <is>
           <t>22.00</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr"/>
+      <c r="L12" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -973,7 +997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1089,64 +1113,71 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>finisaj        – numele finisajului (ex: Poliester mat). Vezi „Valori permise”.</t>
+          <t>producator     – numele producătorului / brandului (ex: Ruukki, Lindab). Opțional. Doar pe primul rând.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>culoare        – numele culorii (ex: Antracit). Lasă gol dacă produsul nu are culori.</t>
+          <t>finisaj        – numele finisajului (ex: Poliester mat). Vezi „Valori permise”.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>grosime        – ex: 0.50 mm. Lasă gol dacă produsul nu are grosimi.</t>
+          <t>culoare        – numele culorii (ex: Antracit). Lasă gol dacă produsul nu are culori.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>pret           – prețul final (lei) al combinației de pe rândul respectiv. Ex: 42.90</t>
+          <t>grosime        – ex: 0.50 mm. Lasă gol dacă produsul nu are grosimi.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
+          <t>pret           – prețul final (lei) al combinației de pe rândul respectiv. Ex: 42.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
           <t>specificatii   – „Cheie: valoare; Cheie: valoare”. Doar pe primul rând.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr"/>
-    </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Sfaturi:</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>• Numele de finisaj/culoare/grosime care nu există încă în tab-ul „Proprietăți” se importă oricum, dar adaugă-le acolo ca să apară numele frumos și pastila de culoare corectă.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>• Poți salva ca .csv (delimitat prin virgulă) și importa la fel.</t>
+          <t>• Numele de finisaj/culoare/grosime care nu există încă în tab-ul „Proprietăți” se importă oricum, dar adaugă-le acolo ca să apară numele frumos și pastila de culoare corectă.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>• Poți salva ca .csv (delimitat prin virgulă) și importa la fel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>• Un produs simplu (fără finisaje) poate fi importat cu formatul vechi: coloane „pret”, „culori”, „pret_culori” în loc de finisaj/culoare/grosime — dar recomandat e formatul de mai sus.</t>
         </is>

</xml_diff>